<commit_message>
added contact matched options
</commit_message>
<xml_diff>
--- a/sample-due-database.xlsx
+++ b/sample-due-database.xlsx
@@ -397,7 +397,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:L29"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="45.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
+    <col min="11" max="11" width="28.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,68 +441,1083 @@
       <c r="I1" t="str">
         <v>Overdue by days</v>
       </c>
+      <c r="J1" t="str">
+        <v>Ageing Days</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Ageing Bucket</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Trigger Rule</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>DLR-001</v>
+        <v>D23057</v>
       </c>
       <c r="B2" t="str">
-        <v>Example Trading Co.</v>
+        <v>A. A. Enterprises</v>
       </c>
       <c r="C2" t="str">
-        <v>INV-1001</v>
+        <v>0629/30.04.2026/P-4/GREASE</v>
       </c>
       <c r="D2" t="str">
-        <v>2026-05-30</v>
+        <v>2026-08-11</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-06-02</v>
+        <v>2026-09-08</v>
       </c>
       <c r="F2">
-        <v>50000</v>
+        <v>152264</v>
       </c>
       <c r="G2">
-        <v>35000</v>
+        <v>147264</v>
       </c>
       <c r="H2" t="str">
         <v>INR</v>
       </c>
       <c r="I2">
-        <v>15</v>
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>28</v>
+      </c>
+      <c r="K2" t="str">
+        <v>25-30 Days (3% CD)</v>
+      </c>
+      <c r="L2" t="str">
+        <v>30 Day Reminder</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>DLR-002</v>
+        <v>D23077</v>
       </c>
       <c r="B3" t="str">
-        <v>Metro Health Supplies</v>
+        <v>Abhijeet Agencies</v>
       </c>
       <c r="C3" t="str">
-        <v>INV-1002</v>
+        <v>5948/31.03.2026/P-1</v>
       </c>
       <c r="D3" t="str">
-        <v>2026-05-03</v>
+        <v>2026-07-28</v>
       </c>
       <c r="E3" t="str">
-        <v>2026-05-18</v>
+        <v>2026-08-27</v>
       </c>
       <c r="F3">
-        <v>42000</v>
+        <v>61399.25</v>
       </c>
       <c r="G3">
-        <v>28000</v>
+        <v>56399.25</v>
       </c>
       <c r="H3" t="str">
         <v>INR</v>
       </c>
       <c r="I3">
-        <v>30</v>
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>42</v>
+      </c>
+      <c r="K3" t="str">
+        <v>40-45 Days (2% CD)</v>
+      </c>
+      <c r="L3" t="str">
+        <v>45 Day Reminder</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>D23119</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Abhijeet Auto Components Private Limited(Nagpur)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>0630/30.04.2026/P-4/GREASE</v>
+      </c>
+      <c r="D4" t="str">
+        <v>2026-07-15</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="F4">
+        <v>72507.8</v>
+      </c>
+      <c r="G4">
+        <v>67507.8</v>
+      </c>
+      <c r="H4" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>55</v>
+      </c>
+      <c r="K4" t="str">
+        <v>50-60 Days (60d Due)</v>
+      </c>
+      <c r="L4" t="str">
+        <v>60 Day Reminder</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>D23119</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Abhijeet Auto Components Private Limited(Nagpur)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>2166/29.06.2026/P-4/GREASE</v>
+      </c>
+      <c r="D5" t="str">
+        <v>2026-07-15</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-08-14</v>
+      </c>
+      <c r="F5">
+        <v>57816.23</v>
+      </c>
+      <c r="G5">
+        <v>52816.23</v>
+      </c>
+      <c r="H5" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>55</v>
+      </c>
+      <c r="K5" t="str">
+        <v>50-60 Days (60d Due)</v>
+      </c>
+      <c r="L5" t="str">
+        <v>60 Day Reminder</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>D23157</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Abhijeet Auto Components Private Limited (Pune)</v>
+      </c>
+      <c r="C6" t="str">
+        <v>0747/21.05.2025/P-1</v>
+      </c>
+      <c r="D6" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="E6" t="str">
+        <v>2026-07-25</v>
+      </c>
+      <c r="F6">
+        <v>11190.32</v>
+      </c>
+      <c r="G6">
+        <v>6190.32</v>
+      </c>
+      <c r="H6" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I6">
+        <v>15</v>
+      </c>
+      <c r="J6">
+        <v>75</v>
+      </c>
+      <c r="K6" t="str">
+        <v>60-90 Days (60+ Overdue)</v>
+      </c>
+      <c r="L6" t="str">
+        <v>75 Day Reminder</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>D23157</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Abhijeet Auto Components Private Limited (Pune)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>1581/15.07.2025/P-1</v>
+      </c>
+      <c r="D7" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="E7" t="str">
+        <v>2026-07-25</v>
+      </c>
+      <c r="F7">
+        <v>10686.14</v>
+      </c>
+      <c r="G7">
+        <v>5686.14</v>
+      </c>
+      <c r="H7" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I7">
+        <v>15</v>
+      </c>
+      <c r="J7">
+        <v>75</v>
+      </c>
+      <c r="K7" t="str">
+        <v>60-90 Days (60+ Overdue)</v>
+      </c>
+      <c r="L7" t="str">
+        <v>75 Day Reminder</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>D23157</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Abhijeet Auto Components Private Limited (Pune)</v>
+      </c>
+      <c r="C8" t="str">
+        <v>3089/16.10.2025/P-1</v>
+      </c>
+      <c r="D8" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="E8" t="str">
+        <v>2026-07-25</v>
+      </c>
+      <c r="F8">
+        <v>25643.78</v>
+      </c>
+      <c r="G8">
+        <v>20643.78</v>
+      </c>
+      <c r="H8" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I8">
+        <v>15</v>
+      </c>
+      <c r="J8">
+        <v>75</v>
+      </c>
+      <c r="K8" t="str">
+        <v>60-90 Days (60+ Overdue)</v>
+      </c>
+      <c r="L8" t="str">
+        <v>75 Day Reminder</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>D23157</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Abhijeet Auto Components Private Limited (Pune)</v>
+      </c>
+      <c r="C9" t="str">
+        <v>4548/06.11.2025/P-4/GREASE</v>
+      </c>
+      <c r="D9" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="E9" t="str">
+        <v>2026-07-25</v>
+      </c>
+      <c r="F9">
+        <v>102029.28</v>
+      </c>
+      <c r="G9">
+        <v>97029.28</v>
+      </c>
+      <c r="H9" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I9">
+        <v>15</v>
+      </c>
+      <c r="J9">
+        <v>75</v>
+      </c>
+      <c r="K9" t="str">
+        <v>60-90 Days (60+ Overdue)</v>
+      </c>
+      <c r="L9" t="str">
+        <v>75 Day Reminder</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>D23157</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Abhijeet Auto Components Private Limited (Pune)</v>
+      </c>
+      <c r="C10" t="str">
+        <v>6384/22.01.2026/P-4/GREASE</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="E10" t="str">
+        <v>2026-07-25</v>
+      </c>
+      <c r="F10">
+        <v>93410.56</v>
+      </c>
+      <c r="G10">
+        <v>88410.56</v>
+      </c>
+      <c r="H10" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I10">
+        <v>15</v>
+      </c>
+      <c r="J10">
+        <v>75</v>
+      </c>
+      <c r="K10" t="str">
+        <v>60-90 Days (60+ Overdue)</v>
+      </c>
+      <c r="L10" t="str">
+        <v>75 Day Reminder</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C11" t="str">
+        <v>0357/15.04.2026/P-4</v>
+      </c>
+      <c r="D11" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E11" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F11">
+        <v>316310.88</v>
+      </c>
+      <c r="G11">
+        <v>83882.69</v>
+      </c>
+      <c r="H11" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I11">
+        <v>45</v>
+      </c>
+      <c r="J11">
+        <v>105</v>
+      </c>
+      <c r="K11" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L11" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C12" t="str">
+        <v>0204/16.04.2026/P-1</v>
+      </c>
+      <c r="D12" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F12">
+        <v>49664.49</v>
+      </c>
+      <c r="G12">
+        <v>44664.49</v>
+      </c>
+      <c r="H12" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I12">
+        <v>45</v>
+      </c>
+      <c r="J12">
+        <v>105</v>
+      </c>
+      <c r="K12" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L12" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C13" t="str">
+        <v>RO/0092</v>
+      </c>
+      <c r="D13" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F13">
+        <v>426249.5</v>
+      </c>
+      <c r="G13">
+        <v>421249.5</v>
+      </c>
+      <c r="H13" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I13">
+        <v>45</v>
+      </c>
+      <c r="J13">
+        <v>105</v>
+      </c>
+      <c r="K13" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L13" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C14" t="str">
+        <v>RO/0093</v>
+      </c>
+      <c r="D14" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F14">
+        <v>264977.6</v>
+      </c>
+      <c r="G14">
+        <v>259977.6</v>
+      </c>
+      <c r="H14" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I14">
+        <v>45</v>
+      </c>
+      <c r="J14">
+        <v>105</v>
+      </c>
+      <c r="K14" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L14" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C15" t="str">
+        <v>0694/12.05.2026/P-2</v>
+      </c>
+      <c r="D15" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E15" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F15">
+        <v>58156.77</v>
+      </c>
+      <c r="G15">
+        <v>53156.77</v>
+      </c>
+      <c r="H15" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I15">
+        <v>45</v>
+      </c>
+      <c r="J15">
+        <v>105</v>
+      </c>
+      <c r="K15" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L15" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C16" t="str">
+        <v>0877/12.05.2026/P-4</v>
+      </c>
+      <c r="D16" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F16">
+        <v>205594.17</v>
+      </c>
+      <c r="G16">
+        <v>200594.17</v>
+      </c>
+      <c r="H16" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I16">
+        <v>45</v>
+      </c>
+      <c r="J16">
+        <v>105</v>
+      </c>
+      <c r="K16" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L16" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C17" t="str">
+        <v>1364/01.06.2026/P-4</v>
+      </c>
+      <c r="D17" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E17" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F17">
+        <v>248456.78</v>
+      </c>
+      <c r="G17">
+        <v>243456.78</v>
+      </c>
+      <c r="H17" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I17">
+        <v>45</v>
+      </c>
+      <c r="J17">
+        <v>105</v>
+      </c>
+      <c r="K17" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L17" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C18" t="str">
+        <v>1008/01.06.2026/P-2</v>
+      </c>
+      <c r="D18" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E18" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F18">
+        <v>124164.12</v>
+      </c>
+      <c r="G18">
+        <v>119164.12</v>
+      </c>
+      <c r="H18" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I18">
+        <v>45</v>
+      </c>
+      <c r="J18">
+        <v>105</v>
+      </c>
+      <c r="K18" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L18" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C19" t="str">
+        <v>RO/0337/03.06.2026</v>
+      </c>
+      <c r="D19" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E19" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F19">
+        <v>264977.6</v>
+      </c>
+      <c r="G19">
+        <v>259977.6</v>
+      </c>
+      <c r="H19" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I19">
+        <v>45</v>
+      </c>
+      <c r="J19">
+        <v>105</v>
+      </c>
+      <c r="K19" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L19" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C20" t="str">
+        <v>RO/0338/03.06.2026</v>
+      </c>
+      <c r="D20" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E20" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F20">
+        <v>18165.57</v>
+      </c>
+      <c r="G20">
+        <v>13165.57</v>
+      </c>
+      <c r="H20" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I20">
+        <v>45</v>
+      </c>
+      <c r="J20">
+        <v>105</v>
+      </c>
+      <c r="K20" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L20" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C21" t="str">
+        <v>2174/29.06.2026/P-4</v>
+      </c>
+      <c r="D21" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E21" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F21">
+        <v>321007.79</v>
+      </c>
+      <c r="G21">
+        <v>316007.79</v>
+      </c>
+      <c r="H21" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I21">
+        <v>45</v>
+      </c>
+      <c r="J21">
+        <v>105</v>
+      </c>
+      <c r="K21" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L21" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>D23278</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Afiya Tractor Parts</v>
+      </c>
+      <c r="C22" t="str">
+        <v>1520/29.06.2026/P-2</v>
+      </c>
+      <c r="D22" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="E22" t="str">
+        <v>2026-06-25</v>
+      </c>
+      <c r="F22">
+        <v>125357.13</v>
+      </c>
+      <c r="G22">
+        <v>120357.13</v>
+      </c>
+      <c r="H22" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I22">
+        <v>45</v>
+      </c>
+      <c r="J22">
+        <v>105</v>
+      </c>
+      <c r="K22" t="str">
+        <v>90-120 Days (90+ Overdue)</v>
+      </c>
+      <c r="L22" t="str">
+        <v>90 Day Reminder</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>D23292</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Allahabad Auto Centre</v>
+      </c>
+      <c r="C23" t="str">
+        <v>1677/12.06.2026/P-4/CLUTCH</v>
+      </c>
+      <c r="D23" t="str">
+        <v>2026-04-26</v>
+      </c>
+      <c r="E23" t="str">
+        <v>2026-05-26</v>
+      </c>
+      <c r="F23">
+        <v>56963.02</v>
+      </c>
+      <c r="G23">
+        <v>51963.02</v>
+      </c>
+      <c r="H23" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I23">
+        <v>75</v>
+      </c>
+      <c r="J23">
+        <v>135</v>
+      </c>
+      <c r="K23" t="str">
+        <v>120+ Days (&gt;120 Overdue)</v>
+      </c>
+      <c r="L23" t="str">
+        <v>120 Day Reminder</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>D23365</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Aman Spare Parts</v>
+      </c>
+      <c r="C24" t="str">
+        <v>3609/24.09.2025/P-4/GREASE</v>
+      </c>
+      <c r="D24" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="E24" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="F24">
+        <v>17885.440000000002</v>
+      </c>
+      <c r="G24">
+        <v>12885.44</v>
+      </c>
+      <c r="H24" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>27</v>
+      </c>
+      <c r="K24" t="str">
+        <v>25-30 Days (3% CD)</v>
+      </c>
+      <c r="L24" t="str">
+        <v>30 Day Reminder</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>D23365</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Aman Spare Parts</v>
+      </c>
+      <c r="C25" t="str">
+        <v>CREDIT NOTE NO. 094/P-4</v>
+      </c>
+      <c r="D25" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="E25" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="F25">
+        <v>20000</v>
+      </c>
+      <c r="G25">
+        <v>15000</v>
+      </c>
+      <c r="H25" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>27</v>
+      </c>
+      <c r="K25" t="str">
+        <v>25-30 Days (3% CD)</v>
+      </c>
+      <c r="L25" t="str">
+        <v>30 Day Reminder</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>D23365</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Aman Spare Parts</v>
+      </c>
+      <c r="C26" t="str">
+        <v>0971/16.05.2026/P-4/GREASE</v>
+      </c>
+      <c r="D26" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="E26" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="F26">
+        <v>156736.44</v>
+      </c>
+      <c r="G26">
+        <v>151736.44</v>
+      </c>
+      <c r="H26" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>27</v>
+      </c>
+      <c r="K26" t="str">
+        <v>25-30 Days (3% CD)</v>
+      </c>
+      <c r="L26" t="str">
+        <v>30 Day Reminder</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>D23365</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Aman Spare Parts</v>
+      </c>
+      <c r="C27" t="str">
+        <v>30.06.2026</v>
+      </c>
+      <c r="D27" t="str">
+        <v>2026-08-12</v>
+      </c>
+      <c r="E27" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="F27">
+        <v>20000</v>
+      </c>
+      <c r="G27">
+        <v>15000</v>
+      </c>
+      <c r="H27" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>27</v>
+      </c>
+      <c r="K27" t="str">
+        <v>25-30 Days (3% CD)</v>
+      </c>
+      <c r="L27" t="str">
+        <v>30 Day Reminder</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>D23469</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Aman Tradings</v>
+      </c>
+      <c r="C28" t="str">
+        <v>6903/16.02.2026/P-4/GREASE</v>
+      </c>
+      <c r="D28" t="str">
+        <v>2026-07-27</v>
+      </c>
+      <c r="E28" t="str">
+        <v>2026-08-26</v>
+      </c>
+      <c r="F28">
+        <v>41674.4</v>
+      </c>
+      <c r="G28">
+        <v>36674.4</v>
+      </c>
+      <c r="H28" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>43</v>
+      </c>
+      <c r="K28" t="str">
+        <v>40-45 Days (2% CD)</v>
+      </c>
+      <c r="L28" t="str">
+        <v>45 Day Reminder</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>D23512</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Amar Auto Agencies</v>
+      </c>
+      <c r="C29" t="str">
+        <v>UP/0635/2023-24</v>
+      </c>
+      <c r="D29" t="str">
+        <v>2026-07-12</v>
+      </c>
+      <c r="E29" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="F29">
+        <v>44694</v>
+      </c>
+      <c r="G29">
+        <v>39694</v>
+      </c>
+      <c r="H29" t="str">
+        <v>INR</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>58</v>
+      </c>
+      <c r="K29" t="str">
+        <v>50-60 Days (60d Due)</v>
+      </c>
+      <c r="L29" t="str">
+        <v>60 Day Reminder</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L29"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>